<commit_message>
feat: use activity aliases to improve reading of excel files.
Sometimes the spreadheets contain the wrong name for an activity instead of it's shorform. E.g we expect "snork" put sometimes the sheet may contain "snorkel". Using aliases we can check for these common variations and turn them into the correct form "snorke" --> "snork" without presenting this as an error to the user. Test included to check if there actual incorrect activities in the sheet such as "flying" which is not offered.
</commit_message>
<xml_diff>
--- a/e2e/fixtures/original-format/error-wrong-activities.xlsx
+++ b/e2e/fixtures/original-format/error-wrong-activities.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/darren/Projects/Sherrif Excel Data/Original Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/darren/Projects/NY-Sheriff-Summer-Camp-Scheduler/e2e/fixtures/original-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5891C77D-4DE7-C54E-B825-0120D024CCBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13DE3B9F-0365-4F45-B664-C4BF4E6B53BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="44800" windowHeight="24600" xr2:uid="{80EEC0AD-E250-4EB9-826C-6224A18D2B1D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="249">
   <si>
     <t>Last Name</t>
   </si>
@@ -227,9 +227,6 @@
     <t>Sanchez</t>
   </si>
   <si>
-    <t>Ball</t>
-  </si>
-  <si>
     <t>Alice</t>
   </si>
   <si>
@@ -774,6 +771,18 @@
   </si>
   <si>
     <t>Sarah</t>
+  </si>
+  <si>
+    <t>fBall</t>
+  </si>
+  <si>
+    <t>diving</t>
+  </si>
+  <si>
+    <t>flying</t>
+  </si>
+  <si>
+    <t>praying</t>
   </si>
 </sst>
 </file>
@@ -1287,10 +1296,10 @@
     </row>
     <row r="2" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
@@ -1316,10 +1325,10 @@
     </row>
     <row r="3" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>75</v>
       </c>
       <c r="C3" s="3">
         <v>5</v>
@@ -1345,10 +1354,10 @@
     </row>
     <row r="4" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>77</v>
       </c>
       <c r="C4" s="2">
         <v>8</v>
@@ -1374,10 +1383,10 @@
     </row>
     <row r="5" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>22</v>
@@ -1403,7 +1412,7 @@
     </row>
     <row r="6" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>39</v>
@@ -1432,10 +1441,10 @@
     </row>
     <row r="7" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>81</v>
       </c>
       <c r="C7" s="3">
         <v>11</v>
@@ -1464,7 +1473,7 @@
         <v>62</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C8" s="4">
         <v>9</v>
@@ -1490,10 +1499,10 @@
     </row>
     <row r="9" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>84</v>
       </c>
       <c r="C9" s="6">
         <v>5</v>
@@ -1519,10 +1528,10 @@
     </row>
     <row r="10" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>85</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>86</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>28</v>
@@ -1548,10 +1557,10 @@
     </row>
     <row r="11" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>87</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>88</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>29</v>
@@ -1577,10 +1586,10 @@
     </row>
     <row r="12" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>89</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>90</v>
       </c>
       <c r="C12" s="4">
         <v>4</v>
@@ -1606,10 +1615,10 @@
     </row>
     <row r="13" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>91</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>92</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>30</v>
@@ -1635,10 +1644,10 @@
     </row>
     <row r="14" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C14" s="6">
         <v>2</v>
@@ -1664,10 +1673,10 @@
     </row>
     <row r="15" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C15" s="4">
         <v>9</v>
@@ -1693,10 +1702,10 @@
     </row>
     <row r="16" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>95</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>96</v>
       </c>
       <c r="C16" s="4">
         <v>1</v>
@@ -1722,10 +1731,10 @@
     </row>
     <row r="17" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>97</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>98</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>34</v>
@@ -1751,10 +1760,10 @@
     </row>
     <row r="18" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>99</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>100</v>
       </c>
       <c r="C18" s="6">
         <v>5</v>
@@ -1780,10 +1789,10 @@
     </row>
     <row r="19" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>102</v>
       </c>
       <c r="C19" s="4">
         <v>1</v>
@@ -1809,10 +1818,10 @@
     </row>
     <row r="20" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>103</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>104</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>38</v>
@@ -1838,10 +1847,10 @@
     </row>
     <row r="21" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>28</v>
@@ -1867,10 +1876,10 @@
     </row>
     <row r="22" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>106</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>107</v>
       </c>
       <c r="C22" s="4">
         <v>11</v>
@@ -1896,7 +1905,7 @@
     </row>
     <row r="23" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>32</v>
@@ -1928,7 +1937,7 @@
         <v>57</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C24" s="6">
         <v>2</v>
@@ -1954,10 +1963,10 @@
     </row>
     <row r="25" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>110</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>111</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>29</v>
@@ -1983,10 +1992,10 @@
     </row>
     <row r="26" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B26" s="6" t="s">
         <v>112</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>113</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>29</v>
@@ -2012,10 +2021,10 @@
     </row>
     <row r="27" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>114</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>115</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>22</v>
@@ -2041,10 +2050,10 @@
     </row>
     <row r="28" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C28" s="6">
         <v>8</v>
@@ -2070,10 +2079,10 @@
     </row>
     <row r="29" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>117</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>118</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>30</v>
@@ -2099,10 +2108,10 @@
     </row>
     <row r="30" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B30" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>38</v>
@@ -2128,10 +2137,10 @@
     </row>
     <row r="31" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C31" s="6">
         <v>5</v>
@@ -2157,10 +2166,10 @@
     </row>
     <row r="32" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>122</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>123</v>
       </c>
       <c r="C32" s="4">
         <v>3</v>
@@ -2186,10 +2195,10 @@
     </row>
     <row r="33" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B33" s="6" t="s">
         <v>124</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>125</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>30</v>
@@ -2215,10 +2224,10 @@
     </row>
     <row r="34" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B34" s="6" t="s">
         <v>126</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>127</v>
       </c>
       <c r="C34" s="4">
         <v>1</v>
@@ -2244,10 +2253,10 @@
     </row>
     <row r="35" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>128</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>129</v>
       </c>
       <c r="C35" s="6">
         <v>2</v>
@@ -2273,10 +2282,10 @@
     </row>
     <row r="36" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="B36" s="6" t="s">
         <v>130</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>131</v>
       </c>
       <c r="C36" s="4">
         <v>3</v>
@@ -2302,10 +2311,10 @@
     </row>
     <row r="37" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B37" s="7" t="s">
         <v>132</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>133</v>
       </c>
       <c r="C37" s="7" t="s">
         <v>28</v>
@@ -2331,10 +2340,10 @@
     </row>
     <row r="38" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B38" s="4" t="s">
         <v>134</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>135</v>
       </c>
       <c r="C38" s="6">
         <v>5</v>
@@ -2360,10 +2369,10 @@
     </row>
     <row r="39" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C39" s="4">
         <v>3</v>
@@ -2389,10 +2398,10 @@
     </row>
     <row r="40" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B40" s="8" t="s">
         <v>137</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>138</v>
       </c>
       <c r="C40" s="8">
         <v>10</v>
@@ -2418,10 +2427,10 @@
     </row>
     <row r="41" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B41" s="7" t="s">
         <v>139</v>
-      </c>
-      <c r="B41" s="7" t="s">
-        <v>140</v>
       </c>
       <c r="C41" s="7">
         <v>5</v>
@@ -2447,10 +2456,10 @@
     </row>
     <row r="42" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C42" s="6">
         <v>2</v>
@@ -2476,10 +2485,10 @@
     </row>
     <row r="43" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B43" s="7" t="s">
         <v>142</v>
-      </c>
-      <c r="B43" s="7" t="s">
-        <v>143</v>
       </c>
       <c r="C43" s="7">
         <v>1</v>
@@ -2505,10 +2514,10 @@
     </row>
     <row r="44" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C44" s="4">
         <v>10</v>
@@ -2534,10 +2543,10 @@
     </row>
     <row r="45" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="B45" s="6" t="s">
         <v>145</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>146</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>34</v>
@@ -2563,10 +2572,10 @@
     </row>
     <row r="46" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A46" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B46" s="8" t="s">
         <v>147</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>148</v>
       </c>
       <c r="C46" s="8">
         <v>2</v>
@@ -2592,7 +2601,7 @@
     </row>
     <row r="47" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>24</v>
@@ -2621,10 +2630,10 @@
     </row>
     <row r="48" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="B48" s="6" t="s">
         <v>149</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>150</v>
       </c>
       <c r="C48" s="6" t="s">
         <v>28</v>
@@ -2650,10 +2659,10 @@
     </row>
     <row r="49" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C49" s="4">
         <v>8</v>
@@ -2679,10 +2688,10 @@
     </row>
     <row r="50" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="B50" s="6" t="s">
         <v>152</v>
-      </c>
-      <c r="B50" s="6" t="s">
-        <v>153</v>
       </c>
       <c r="C50" s="6">
         <v>10</v>
@@ -2708,10 +2717,10 @@
     </row>
     <row r="51" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="B51" s="6" t="s">
         <v>154</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>155</v>
       </c>
       <c r="C51" s="6">
         <v>10</v>
@@ -2737,10 +2746,10 @@
     </row>
     <row r="52" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C52" s="7">
         <v>11</v>
@@ -2766,10 +2775,10 @@
     </row>
     <row r="53" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>30</v>
@@ -2795,10 +2804,10 @@
     </row>
     <row r="54" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B54" s="4" t="s">
         <v>158</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>159</v>
       </c>
       <c r="C54" s="4">
         <v>3</v>
@@ -2824,10 +2833,10 @@
     </row>
     <row r="55" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B55" s="4" t="s">
         <v>160</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>161</v>
       </c>
       <c r="C55" s="4">
         <v>2</v>
@@ -2853,10 +2862,10 @@
     </row>
     <row r="56" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B56" s="4" t="s">
         <v>162</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>163</v>
       </c>
       <c r="C56" s="6">
         <v>1</v>
@@ -2882,10 +2891,10 @@
     </row>
     <row r="57" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="B57" s="6" t="s">
         <v>164</v>
-      </c>
-      <c r="B57" s="6" t="s">
-        <v>165</v>
       </c>
       <c r="C57" s="4">
         <v>10</v>
@@ -2911,7 +2920,7 @@
     </row>
     <row r="58" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>40</v>
@@ -2940,10 +2949,10 @@
     </row>
     <row r="59" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>9</v>
@@ -2969,10 +2978,10 @@
     </row>
     <row r="60" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="B60" s="6" t="s">
         <v>168</v>
-      </c>
-      <c r="B60" s="6" t="s">
-        <v>169</v>
       </c>
       <c r="C60" s="6">
         <v>3</v>
@@ -2998,10 +3007,10 @@
     </row>
     <row r="61" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B61" s="4" t="s">
         <v>170</v>
-      </c>
-      <c r="B61" s="4" t="s">
-        <v>171</v>
       </c>
       <c r="C61" s="4">
         <v>11</v>
@@ -3027,10 +3036,10 @@
     </row>
     <row r="62" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B62" s="4" t="s">
         <v>172</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>173</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>29</v>
@@ -3056,10 +3065,10 @@
     </row>
     <row r="63" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B63" s="4" t="s">
         <v>174</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>175</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>28</v>
@@ -3088,7 +3097,7 @@
         <v>32</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>22</v>
@@ -3114,10 +3123,10 @@
     </row>
     <row r="65" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>30</v>
@@ -3143,10 +3152,10 @@
     </row>
     <row r="66" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B66" s="4" t="s">
         <v>178</v>
-      </c>
-      <c r="B66" s="4" t="s">
-        <v>179</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>9</v>
@@ -3172,7 +3181,7 @@
     </row>
     <row r="67" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B67" s="7" t="s">
         <v>41</v>
@@ -3201,10 +3210,10 @@
     </row>
     <row r="68" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="B68" s="6" t="s">
         <v>181</v>
-      </c>
-      <c r="B68" s="6" t="s">
-        <v>182</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>34</v>
@@ -3230,10 +3239,10 @@
     </row>
     <row r="69" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="B69" s="7" t="s">
         <v>183</v>
-      </c>
-      <c r="B69" s="7" t="s">
-        <v>184</v>
       </c>
       <c r="C69" s="7">
         <v>11</v>
@@ -3262,7 +3271,7 @@
         <v>31</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>28</v>
@@ -3288,10 +3297,10 @@
     </row>
     <row r="71" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="B71" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="B71" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>38</v>
@@ -3317,10 +3326,10 @@
     </row>
     <row r="72" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="B72" s="7" t="s">
         <v>188</v>
-      </c>
-      <c r="B72" s="7" t="s">
-        <v>189</v>
       </c>
       <c r="C72" s="7">
         <v>3</v>
@@ -3346,10 +3355,10 @@
     </row>
     <row r="73" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B73" s="8" t="s">
         <v>190</v>
-      </c>
-      <c r="B73" s="8" t="s">
-        <v>191</v>
       </c>
       <c r="C73" s="8">
         <v>4</v>
@@ -3375,10 +3384,10 @@
     </row>
     <row r="74" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="B74" s="7" t="s">
         <v>192</v>
-      </c>
-      <c r="B74" s="7" t="s">
-        <v>193</v>
       </c>
       <c r="C74" s="7">
         <v>2</v>
@@ -3404,10 +3413,10 @@
     </row>
     <row r="75" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B75" s="6" t="s">
         <v>194</v>
-      </c>
-      <c r="B75" s="6" t="s">
-        <v>195</v>
       </c>
       <c r="C75" s="6" t="s">
         <v>29</v>
@@ -3433,7 +3442,7 @@
     </row>
     <row r="76" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A76" s="7" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B76" s="7" t="s">
         <v>42</v>
@@ -3448,7 +3457,7 @@
         <v>55</v>
       </c>
       <c r="F76" s="7" t="s">
-        <v>63</v>
+        <v>245</v>
       </c>
       <c r="G76" s="7" t="s">
         <v>53</v>
@@ -3462,10 +3471,10 @@
     </row>
     <row r="77" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="B77" s="8" t="s">
         <v>197</v>
-      </c>
-      <c r="B77" s="8" t="s">
-        <v>198</v>
       </c>
       <c r="C77" s="8">
         <v>9</v>
@@ -3491,10 +3500,10 @@
     </row>
     <row r="78" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A78" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B78" s="7" t="s">
         <v>199</v>
-      </c>
-      <c r="B78" s="7" t="s">
-        <v>200</v>
       </c>
       <c r="C78" s="7">
         <v>4</v>
@@ -3520,10 +3529,10 @@
     </row>
     <row r="79" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="B79" s="8" t="s">
         <v>201</v>
-      </c>
-      <c r="B79" s="8" t="s">
-        <v>202</v>
       </c>
       <c r="C79" s="8">
         <v>8</v>
@@ -3549,10 +3558,10 @@
     </row>
     <row r="80" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A80" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="B80" s="7" t="s">
         <v>203</v>
-      </c>
-      <c r="B80" s="7" t="s">
-        <v>204</v>
       </c>
       <c r="C80" s="7" t="s">
         <v>34</v>
@@ -3578,7 +3587,7 @@
     </row>
     <row r="81" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B81" s="7" t="s">
         <v>42</v>
@@ -3596,7 +3605,7 @@
         <v>23</v>
       </c>
       <c r="G81" s="7" t="s">
-        <v>21</v>
+        <v>248</v>
       </c>
       <c r="H81" s="7" t="s">
         <v>19</v>
@@ -3607,10 +3616,10 @@
     </row>
     <row r="82" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A82" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="B82" s="7" t="s">
         <v>206</v>
-      </c>
-      <c r="B82" s="7" t="s">
-        <v>207</v>
       </c>
       <c r="C82" s="7" t="s">
         <v>29</v>
@@ -3636,10 +3645,10 @@
     </row>
     <row r="83" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="B83" s="8" t="s">
         <v>208</v>
-      </c>
-      <c r="B83" s="8" t="s">
-        <v>209</v>
       </c>
       <c r="C83" s="8" t="s">
         <v>9</v>
@@ -3665,10 +3674,10 @@
     </row>
     <row r="84" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A84" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="B84" s="7" t="s">
         <v>210</v>
-      </c>
-      <c r="B84" s="7" t="s">
-        <v>211</v>
       </c>
       <c r="C84" s="7">
         <v>4</v>
@@ -3694,10 +3703,10 @@
     </row>
     <row r="85" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="B85" s="8" t="s">
         <v>212</v>
-      </c>
-      <c r="B85" s="8" t="s">
-        <v>213</v>
       </c>
       <c r="C85" s="8">
         <v>9</v>
@@ -3723,10 +3732,10 @@
     </row>
     <row r="86" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A86" s="7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B86" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C86" s="7">
         <v>4</v>
@@ -3752,10 +3761,10 @@
     </row>
     <row r="87" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B87" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C87" s="8" t="s">
         <v>22</v>
@@ -3784,7 +3793,7 @@
         <v>59</v>
       </c>
       <c r="B88" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C88" s="8">
         <v>4</v>
@@ -3813,7 +3822,7 @@
         <v>33</v>
       </c>
       <c r="B89" s="7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C89" s="7">
         <v>11</v>
@@ -3839,10 +3848,10 @@
     </row>
     <row r="90" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A90" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="B90" s="8" t="s">
         <v>217</v>
-      </c>
-      <c r="B90" s="8" t="s">
-        <v>218</v>
       </c>
       <c r="C90" s="8">
         <v>10</v>
@@ -3868,10 +3877,10 @@
     </row>
     <row r="91" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B91" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C91" s="7" t="s">
         <v>9</v>
@@ -3897,7 +3906,7 @@
     </row>
     <row r="92" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A92" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B92" s="8" t="s">
         <v>24</v>
@@ -3926,10 +3935,10 @@
     </row>
     <row r="93" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="B93" s="7" t="s">
         <v>221</v>
-      </c>
-      <c r="B93" s="7" t="s">
-        <v>222</v>
       </c>
       <c r="C93" s="7" t="s">
         <v>34</v>
@@ -3955,10 +3964,10 @@
     </row>
     <row r="94" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A94" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="B94" s="8" t="s">
         <v>223</v>
-      </c>
-      <c r="B94" s="8" t="s">
-        <v>224</v>
       </c>
       <c r="C94" s="8" t="s">
         <v>38</v>
@@ -3984,10 +3993,10 @@
     </row>
     <row r="95" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="B95" s="7" t="s">
         <v>225</v>
-      </c>
-      <c r="B95" s="7" t="s">
-        <v>226</v>
       </c>
       <c r="C95" s="7">
         <v>4</v>
@@ -4013,10 +4022,10 @@
     </row>
     <row r="96" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A96" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="B96" s="7" t="s">
         <v>227</v>
-      </c>
-      <c r="B96" s="7" t="s">
-        <v>228</v>
       </c>
       <c r="C96" s="7">
         <v>9</v>
@@ -4042,10 +4051,10 @@
     </row>
     <row r="97" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="B97" s="8" t="s">
         <v>229</v>
-      </c>
-      <c r="B97" s="8" t="s">
-        <v>230</v>
       </c>
       <c r="C97" s="8">
         <v>10</v>
@@ -4054,7 +4063,7 @@
         <v>56</v>
       </c>
       <c r="E97" s="8" t="s">
-        <v>58</v>
+        <v>247</v>
       </c>
       <c r="F97" s="8" t="s">
         <v>55</v>
@@ -4071,10 +4080,10 @@
     </row>
     <row r="98" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A98" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="B98" s="7" t="s">
         <v>231</v>
-      </c>
-      <c r="B98" s="7" t="s">
-        <v>232</v>
       </c>
       <c r="C98" s="7" t="s">
         <v>9</v>
@@ -4100,10 +4109,10 @@
     </row>
     <row r="99" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B99" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C99" s="8" t="s">
         <v>22</v>
@@ -4129,10 +4138,10 @@
     </row>
     <row r="100" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A100" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="B100" s="7" t="s">
         <v>234</v>
-      </c>
-      <c r="B100" s="7" t="s">
-        <v>235</v>
       </c>
       <c r="C100" s="7" t="s">
         <v>22</v>
@@ -4158,10 +4167,10 @@
     </row>
     <row r="101" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="B101" s="8" t="s">
         <v>236</v>
-      </c>
-      <c r="B101" s="8" t="s">
-        <v>237</v>
       </c>
       <c r="C101" s="8">
         <v>11</v>
@@ -4187,10 +4196,10 @@
     </row>
     <row r="102" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A102" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B102" s="7" t="s">
         <v>238</v>
-      </c>
-      <c r="B102" s="7" t="s">
-        <v>239</v>
       </c>
       <c r="C102" s="7" t="s">
         <v>9</v>
@@ -4216,10 +4225,10 @@
     </row>
     <row r="103" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="B103" s="8" t="s">
         <v>240</v>
-      </c>
-      <c r="B103" s="8" t="s">
-        <v>241</v>
       </c>
       <c r="C103" s="8" t="s">
         <v>29</v>
@@ -4228,10 +4237,10 @@
         <v>56</v>
       </c>
       <c r="E103" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F103" s="8" t="s">
-        <v>44</v>
+        <v>246</v>
       </c>
       <c r="G103" s="8" t="s">
         <v>46</v>
@@ -4245,10 +4254,10 @@
     </row>
     <row r="104" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A104" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="B104" s="7" t="s">
         <v>242</v>
-      </c>
-      <c r="B104" s="7" t="s">
-        <v>243</v>
       </c>
       <c r="C104" s="7">
         <v>1</v>
@@ -4274,10 +4283,10 @@
     </row>
     <row r="105" spans="1:9" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A105" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="B105" s="8" t="s">
         <v>244</v>
-      </c>
-      <c r="B105" s="8" t="s">
-        <v>245</v>
       </c>
       <c r="C105" s="8">
         <v>5</v>

</xml_diff>